<commit_message>
docs(report): update 12-quarter master Excel and PDF report with dynamic concurrent margin recycling & Rs text font rendering
</commit_message>
<xml_diff>
--- a/Nifty50_12_Quarters_Detailed_TradeLog_Master.xlsx
+++ b/Nifty50_12_Quarters_Detailed_TradeLog_Master.xlsx
@@ -585,17 +585,17 @@
   <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="118" customWidth="1" min="1" max="1"/>
+    <col width="97" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -608,7 +608,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Audited Performance Summary across 12 Completed Quarters (Oct 2023 - Sep 2026) with 0.05% Futures Transaction Cost</t>
+          <t>Dynamic Day-by-Day Peak Margin Recycling &amp; 0.05% Futures Transaction Cost Audited Performance</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Overall Win Rate %</t>
+          <t>Overall Net Win Rate %</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
@@ -683,31 +683,31 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Average Fund Utilised / Margin per Quarter</t>
+          <t>Average Peak Fund Utilised / Margin per Quarter</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>13956442.66666667</v>
+        <v>5689782.333333333</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Average Net Return on Fund Utilised % (per Quarter)</t>
+          <t>Average Net Return on Peak Fund Utilised % (per Quarter)</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.05002417356702074</v>
+        <v>0.122704080654434</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Annualized Return on Utilised Fund (CAGR)</t>
+          <t>Annualized Return on Peak Utilised Fund (CAGR)</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.2000966942680831</v>
+        <v>0.4215</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>💰 DYNAMIC 12-QUARTER FUND ALLOCATION &amp; PERFORMANCE BREAKDOWN</t>
+          <t>💰 DYNAMIC 12-QUARTER RECYCLED FUND ALLOCATION &amp; PERFORMANCE BREAKDOWN</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Fund Utilised (Margin ₹)</t>
+          <t>Peak Fund Utilised (Margin ₹)</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>Return on Fund Utilised %</t>
+          <t>Return on Peak Fund %</t>
         </is>
       </c>
     </row>
@@ -810,19 +810,19 @@
         <v>0.86</v>
       </c>
       <c r="G19" s="15" t="n">
-        <v>13927117</v>
+        <v>8701672</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>1409809</v>
       </c>
       <c r="I19" s="15" t="n">
-        <v>36583.70665608855</v>
+        <v>36583.70665608857</v>
       </c>
       <c r="J19" s="16" t="n">
         <v>1373225.293343911</v>
       </c>
       <c r="K19" s="14" t="n">
-        <v>0.09860082983031675</v>
+        <v>0.1578116588793408</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
@@ -849,19 +849,19 @@
         <v>0.6</v>
       </c>
       <c r="G20" s="15" t="n">
-        <v>13927117</v>
+        <v>4290246</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>546340</v>
       </c>
       <c r="I20" s="15" t="n">
-        <v>36170.79370561593</v>
+        <v>36170.79370561592</v>
       </c>
       <c r="J20" s="16" t="n">
         <v>510169.2062943841</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>0.03663135782476618</v>
+        <v>0.1189137420778165</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
@@ -888,19 +888,19 @@
         <v>0.72</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>13927117</v>
+        <v>4955407</v>
       </c>
       <c r="H21" s="15" t="n">
         <v>1019043</v>
       </c>
       <c r="I21" s="15" t="n">
-        <v>36627.08812018742</v>
+        <v>36627.08812018741</v>
       </c>
       <c r="J21" s="16" t="n">
-        <v>982415.9118798128</v>
+        <v>982415.9118798126</v>
       </c>
       <c r="K21" s="14" t="n">
-        <v>0.07053979024372473</v>
+        <v>0.1982513064779164</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -927,7 +927,7 @@
         <v>0.66</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>13927117</v>
+        <v>5376772</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>504453</v>
@@ -939,7 +939,7 @@
         <v>467667.3911225823</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>0.03357962679013771</v>
+        <v>0.0869792118993668</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
@@ -966,19 +966,19 @@
         <v>0.5102040816326531</v>
       </c>
       <c r="G23" s="15" t="n">
-        <v>13880469</v>
+        <v>6818828</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>30263</v>
       </c>
       <c r="I23" s="15" t="n">
-        <v>34527.17005867519</v>
+        <v>34527.1700586752</v>
       </c>
       <c r="J23" s="17" t="n">
-        <v>-4264.170058675183</v>
+        <v>-4264.170058675176</v>
       </c>
       <c r="K23" s="18" t="n">
-        <v>-0.0003072064826249879</v>
+        <v>-0.0006253523418797446</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
@@ -1005,19 +1005,19 @@
         <v>0.62</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>13927117</v>
+        <v>3864500</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>643157</v>
       </c>
       <c r="I24" s="15" t="n">
-        <v>33902.81806275016</v>
+        <v>33902.81806275017</v>
       </c>
       <c r="J24" s="16" t="n">
         <v>609254.1819372498</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>0.04374589385134409</v>
+        <v>0.157654077354703</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
@@ -1044,7 +1044,7 @@
         <v>0.52</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>13927117</v>
+        <v>4740100</v>
       </c>
       <c r="H25" s="15" t="n">
         <v>133872</v>
@@ -1056,7 +1056,7 @@
         <v>100403.4882419074</v>
       </c>
       <c r="K25" s="14" t="n">
-        <v>0.007209208355319155</v>
+        <v>0.0211817236433635</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
@@ -1083,7 +1083,7 @@
         <v>0.62</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>13927117</v>
+        <v>5205794</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>421894</v>
@@ -1095,7 +1095,7 @@
         <v>385898.498144918</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>0.02770842652825549</v>
+        <v>0.0741286532169575</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
@@ -1122,19 +1122,19 @@
         <v>0.68</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>13927117</v>
+        <v>4460297</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>884374</v>
       </c>
       <c r="I27" s="15" t="n">
-        <v>35053.6415488572</v>
+        <v>35053.64154885719</v>
       </c>
       <c r="J27" s="16" t="n">
-        <v>849320.358451143</v>
+        <v>849320.3584511428</v>
       </c>
       <c r="K27" s="14" t="n">
-        <v>0.06098321414626897</v>
+        <v>0.1904178933490624</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
@@ -1161,7 +1161,7 @@
         <v>0.6666666666666665</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>14077117</v>
+        <v>5592565</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>539612</v>
@@ -1170,10 +1170,10 @@
         <v>33279.58137179321</v>
       </c>
       <c r="J28" s="16" t="n">
-        <v>506332.4186282069</v>
+        <v>506332.4186282068</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>0.03596847412919896</v>
+        <v>0.09053670697224024</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
@@ -1200,19 +1200,19 @@
         <v>0.9607843137254902</v>
       </c>
       <c r="G29" s="15" t="n">
-        <v>14077117</v>
+        <v>7172701</v>
       </c>
       <c r="H29" s="15" t="n">
         <v>1864360</v>
       </c>
       <c r="I29" s="15" t="n">
-        <v>31249.10261961177</v>
+        <v>31249.10261961178</v>
       </c>
       <c r="J29" s="16" t="n">
-        <v>1833110.897380389</v>
+        <v>1833110.897380388</v>
       </c>
       <c r="K29" s="14" t="n">
-        <v>0.130219198816092</v>
+        <v>0.255567727886662</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
@@ -1239,19 +1239,19 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="G30" s="15" t="n">
-        <v>14025673</v>
+        <v>7098506</v>
       </c>
       <c r="H30" s="15" t="n">
         <v>790647</v>
       </c>
       <c r="I30" s="15" t="n">
-        <v>26266.35133974351</v>
+        <v>26266.35133974352</v>
       </c>
       <c r="J30" s="16" t="n">
-        <v>764380.6486602563</v>
+        <v>764380.6486602565</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>0.05449867886270101</v>
+        <v>0.1076819049896213</v>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
@@ -1278,7 +1278,7 @@
         <v>0.697171381031614</v>
       </c>
       <c r="G31" s="22" t="n">
-        <v>13956442.66666667</v>
+        <v>5689782.333333333</v>
       </c>
       <c r="H31" s="22" t="n">
         <v>8787824</v>
@@ -1290,7 +1290,7 @@
         <v>8377914.124026085</v>
       </c>
       <c r="K31" s="21" t="n">
-        <v>0.0005002417356702074</v>
+        <v>0.122704080654434</v>
       </c>
     </row>
   </sheetData>
@@ -1313,7 +1313,7 @@
   <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="125" customWidth="1" min="1" max="1"/>
+    <col width="149" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -1344,7 +1344,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 50 | Wins: 34 | Losses: 16 | Win Rate: 68.0% | Fund Utilised: ₹13,927,117.00 | Net Realized PnL: ₹849,320.36</t>
+          <t>Trades: 50 | Wins: 34 | Losses: 16 | Win Rate: 68.0% | Peak Fund Utilised: ₹4,460,297.00 | Net Realized PnL: ₹849,320.36 | Net Ret on Fund: 19.04%</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
   <dimension ref="A1:S55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="125" customWidth="1" min="1" max="1"/>
+    <col width="148" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -5245,7 +5245,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 51 | Wins: 34 | Losses: 17 | Win Rate: 66.7% | Fund Utilised: ₹14,077,117.00 | Net Realized PnL: ₹506,332.42</t>
+          <t>Trades: 51 | Wins: 34 | Losses: 17 | Win Rate: 66.7% | Peak Fund Utilised: ₹5,592,565.00 | Net Realized PnL: ₹506,332.42 | Net Ret on Fund: 9.05%</t>
         </is>
       </c>
     </row>
@@ -9190,7 +9190,7 @@
   <dimension ref="A1:S55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="126" customWidth="1" min="1" max="1"/>
+    <col width="150" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -9221,7 +9221,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 51 | Wins: 49 | Losses: 2 | Win Rate: 96.1% | Fund Utilised: ₹14,077,117.00 | Net Realized PnL: ₹1,833,110.90</t>
+          <t>Trades: 51 | Wins: 49 | Losses: 2 | Win Rate: 96.1% | Peak Fund Utilised: ₹7,172,701.00 | Net Realized PnL: ₹1,833,110.90 | Net Ret on Fund: 25.56%</t>
         </is>
       </c>
     </row>
@@ -13166,7 +13166,7 @@
   <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="124" customWidth="1" min="1" max="1"/>
+    <col width="148" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -13197,7 +13197,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 50 | Wins: 47 | Losses: 3 | Win Rate: 94.0% | Fund Utilised: ₹14,025,673.00 | Net Realized PnL: ₹764,380.65</t>
+          <t>Trades: 50 | Wins: 47 | Losses: 3 | Win Rate: 94.0% | Peak Fund Utilised: ₹7,098,506.00 | Net Realized PnL: ₹764,380.65 | Net Ret on Fund: 10.77%</t>
         </is>
       </c>
     </row>
@@ -17067,7 +17067,7 @@
   <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="126" customWidth="1" min="1" max="1"/>
+    <col width="150" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -17098,7 +17098,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 50 | Wins: 43 | Losses: 7 | Win Rate: 86.0% | Fund Utilised: ₹13,927,117.00 | Net Realized PnL: ₹1,373,225.29</t>
+          <t>Trades: 50 | Wins: 43 | Losses: 7 | Win Rate: 86.0% | Peak Fund Utilised: ₹8,701,672.00 | Net Realized PnL: ₹1,373,225.29 | Net Ret on Fund: 15.78%</t>
         </is>
       </c>
     </row>
@@ -20968,7 +20968,7 @@
   <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="125" customWidth="1" min="1" max="1"/>
+    <col width="149" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -20999,7 +20999,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 50 | Wins: 30 | Losses: 20 | Win Rate: 60.0% | Fund Utilised: ₹13,927,117.00 | Net Realized PnL: ₹510,169.21</t>
+          <t>Trades: 50 | Wins: 30 | Losses: 20 | Win Rate: 60.0% | Peak Fund Utilised: ₹4,290,246.00 | Net Realized PnL: ₹510,169.21 | Net Ret on Fund: 11.89%</t>
         </is>
       </c>
     </row>
@@ -24869,7 +24869,7 @@
   <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="125" customWidth="1" min="1" max="1"/>
+    <col width="149" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -24900,7 +24900,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 50 | Wins: 36 | Losses: 14 | Win Rate: 72.0% | Fund Utilised: ₹13,927,117.00 | Net Realized PnL: ₹982,415.91</t>
+          <t>Trades: 50 | Wins: 36 | Losses: 14 | Win Rate: 72.0% | Peak Fund Utilised: ₹4,955,407.00 | Net Realized PnL: ₹982,415.91 | Net Ret on Fund: 19.83%</t>
         </is>
       </c>
     </row>
@@ -28770,7 +28770,7 @@
   <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="125" customWidth="1" min="1" max="1"/>
+    <col width="148" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -28801,7 +28801,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 50 | Wins: 33 | Losses: 17 | Win Rate: 66.0% | Fund Utilised: ₹13,927,117.00 | Net Realized PnL: ₹467,667.39</t>
+          <t>Trades: 50 | Wins: 33 | Losses: 17 | Win Rate: 66.0% | Peak Fund Utilised: ₹5,376,772.00 | Net Realized PnL: ₹467,667.39 | Net Ret on Fund: 8.70%</t>
         </is>
       </c>
     </row>
@@ -32671,7 +32671,7 @@
   <dimension ref="A1:S53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="124" customWidth="1" min="1" max="1"/>
+    <col width="148" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -32702,7 +32702,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 49 | Wins: 25 | Losses: 24 | Win Rate: 51.0% | Fund Utilised: ₹13,880,469.00 | Net Realized PnL: ₹-4,264.17</t>
+          <t>Trades: 49 | Wins: 25 | Losses: 24 | Win Rate: 51.0% | Peak Fund Utilised: ₹6,818,828.00 | Net Realized PnL: ₹-4,264.17 | Net Ret on Fund: -0.06%</t>
         </is>
       </c>
     </row>
@@ -36497,7 +36497,7 @@
   <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="125" customWidth="1" min="1" max="1"/>
+    <col width="149" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -36528,7 +36528,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 50 | Wins: 31 | Losses: 19 | Win Rate: 62.0% | Fund Utilised: ₹13,927,117.00 | Net Realized PnL: ₹609,254.18</t>
+          <t>Trades: 50 | Wins: 31 | Losses: 19 | Win Rate: 62.0% | Peak Fund Utilised: ₹3,864,500.00 | Net Realized PnL: ₹609,254.18 | Net Ret on Fund: 15.77%</t>
         </is>
       </c>
     </row>
@@ -40398,7 +40398,7 @@
   <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="125" customWidth="1" min="1" max="1"/>
+    <col width="148" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -40429,7 +40429,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 50 | Wins: 26 | Losses: 24 | Win Rate: 52.0% | Fund Utilised: ₹13,927,117.00 | Net Realized PnL: ₹100,403.49</t>
+          <t>Trades: 50 | Wins: 26 | Losses: 24 | Win Rate: 52.0% | Peak Fund Utilised: ₹4,740,100.00 | Net Realized PnL: ₹100,403.49 | Net Ret on Fund: 2.12%</t>
         </is>
       </c>
     </row>
@@ -44299,7 +44299,7 @@
   <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="125" customWidth="1" min="1" max="1"/>
+    <col width="148" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -44330,7 +44330,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Trades: 50 | Wins: 31 | Losses: 19 | Win Rate: 62.0% | Fund Utilised: ₹13,927,117.00 | Net Realized PnL: ₹385,898.50</t>
+          <t>Trades: 50 | Wins: 31 | Losses: 19 | Win Rate: 62.0% | Peak Fund Utilised: ₹5,205,794.00 | Net Realized PnL: ₹385,898.50 | Net Ret on Fund: 7.41%</t>
         </is>
       </c>
     </row>

</xml_diff>